<commit_message>
docs(scorecard): accessibility 72->92; composite 74.1->74.6
VoiceOver Session 3 done (~90%); A1/A2/A3 batches landed;
TODO-TRACKER updated
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1091,7 +1091,7 @@
         <v>2</v>
       </c>
       <c r="G13" s="43" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="H13" s="39">
         <f>IF(G13="","",G13*F13)</f>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="I13" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: Keyboard/a11y pass Sep 12; VoiceOver Session 3 NOT done</t>
+          <t>Sep 14 2026: VoiceOver Session 3 DONE (~90% speak-correct); 0 unnamed buttons repo-wide; 0 generic labels; dialogs trapped+labelled; switch/tab/menu/progressbar roles; accordion expanded states; live regions (shell announcer, alerts, BMI status); inert hidden trees; tour focus restore. Residual: Session 4 UI-look naming, toast-only copy feedback, palette trap, tab arrow-key nav.</t>
         </is>
       </c>
     </row>
@@ -2783,7 +2783,6 @@
         </is>
       </c>
     </row>
-    <row r="56"/>
     <row r="57" ht="15" customHeight="1" s="35">
       <c r="A57" s="52" t="n"/>
       <c r="B57" s="53" t="inlineStr">

</xml_diff>

<commit_message>
docs(scorecard): accessibility 92->95; composite 74.6->74.7
All 9 tab sets complete; worst-offender + duplicate sweeps done;
scans at zero; tsc clean
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1091,7 +1091,7 @@
         <v>2</v>
       </c>
       <c r="G13" s="43" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="H13" s="39">
         <f>IF(G13="","",G13*F13)</f>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="I13" s="40" t="inlineStr">
         <is>
-          <t>Sep 14 2026: VoiceOver Session 3 DONE (~90% speak-correct); 0 unnamed buttons repo-wide; 0 generic labels; dialogs trapped+labelled; switch/tab/menu/progressbar roles; accordion expanded states; live regions (shell announcer, alerts, BMI status); inert hidden trees; tour focus restore. Residual: Session 4 UI-look naming, toast-only copy feedback, palette trap, tab arrow-key nav.</t>
+          <t>Sep 14 2026: 95 — all 9 tab sets complete (shared useRovingTabs hook, panels paired); worst-offender sweep (Copy/Download object-named, single letters expanded, duplicates qualified); unnamed/vague/generic scans all 0; tsc clean; targeted tests 13/13. Residual to 97+: human Session-4 dense-page pass, full-suite CI confirmation on push.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: workbook #14 Testing 85->88 (212 files, 4 E2E + axe gate, Sep 15 evidence)
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1291,7 +1291,7 @@
         <v>2</v>
       </c>
       <c r="G18" s="43" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="H18" s="39">
         <f>IF(G18="","",G18*F18)</f>
@@ -1299,7 +1299,7 @@
       </c>
       <c r="I18" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: 1158 tests: contracts, regression, guards; no E2E yet</t>
+          <t>Sep 15 2026: 212 test files, 4 Playwright E2E (critical/auth/responsive/a11y) + axe gate; 1208/1208 green Sep 14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: #2 70->76, demand-driven batch policy, 30-day structural freeze
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -811,7 +811,7 @@
         <v>3</v>
       </c>
       <c r="G6" s="43" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="H6" s="39">
         <f>IF(G6="","",G6*F6)</f>
@@ -819,7 +819,7 @@
       </c>
       <c r="I6" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: Thin descriptions persist; generic FAQs; honesty fixes Sep 12</t>
+          <t>Sep 15 2026: 49 tools deepened w/ worked-example FAQs + 21 hub intros rewritten; 288/1144 w/ 4+ FAQs; tail 847 zero-custom via fallback (bulk path pending)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: legal row #44 82 -> 96, composite 74.9 -> 75.1
Updates xlsx G48/I48 + scorecard.md log for dca5e782. #26 held at 72
for full Phase 1; see scorecard entry for rationale.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -2491,7 +2491,7 @@
         <v>1</v>
       </c>
       <c r="G48" s="43" t="n">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="H48" s="39">
         <f>IF(G48="","",G48*F48)</f>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="I48" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: Privacy/terms/cookies/disclaimer/security present</t>
+          <t>Sep 16 2026: accuracy pass vs live code (dca5e782) — AI-proxy truth, telemetry disclosed, Decline enforced, Terms dated, Disclaimer re-scoped</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: compliance row #26 72 -> 90, composite 75.1 -> 75.5
Updates xlsx G30/I30 + scorecard.md log for b6055cb0. Held below the
95 target for: unnamed DPDP officer (owner), live prod check, lawyer
review.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1771,7 +1771,7 @@
         <v>2</v>
       </c>
       <c r="G30" s="43" t="n">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="H30" s="39">
         <f>IF(G30="","",G30*F30)</f>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="I30" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: Policy pages present; consent banner not verified</t>
+          <t>Sep 16 2026: banner placebo fixed (Decline gates PostHog/telemetry), policy audited (dca5e782), erasure cascade + 90-day purge enforced (b6055cb0). Residual: unnamed DPDP officer (owner), live prod check, lawyer review</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: privacy-review row #51 55 -> 88, composite 75.5 -> 75.9
Updates xlsx G55/I55 + scorecard.md log for a5d29f27 + 0af1ed3b.
Held below 92 for first real sign-off + PR-template wiring.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -2771,7 +2771,7 @@
         <v>1</v>
       </c>
       <c r="G55" s="43" t="n">
-        <v>55</v>
+        <v>88</v>
       </c>
       <c r="H55" s="39">
         <f>IF(G55="","",G55*F55)</f>
@@ -2779,7 +2779,7 @@
       </c>
       <c r="I55" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: Ad-hoc reviews live, no formal process</t>
+          <t>Sep 16 2026: formalized (a5d29f27) — privacy-gate.test.ts 6/6 in CI + PRIVACY-GATE.md checklist; gate caught 1 real issue on first run. Residual: first real sign-off, PR-template wiring</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: analytics row #34 72 -> 88, composite 75.9 -> 76.3
Updates xlsx G38/I38 + scorecard.md log for 4e5aaf2a. Held below 90
for real-traffic validation + 7d funnel toggle.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -2091,7 +2091,7 @@
         <v>2</v>
       </c>
       <c r="G38" s="43" t="n">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="H38" s="39">
         <f>IF(G38="","",G38*F38)</f>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="I38" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: PostHog + new credit/download events; funnels basic</t>
+          <t>Sep 16 2026: 3 conversion funnels live in admin (4e5aaf2a) + dead Top-tools usedAt fix. Residual: traffic volume for meaningful rates, 7d toggle for funnels</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: data row #27 68 -> 88, composite 76.3 -> 76.8
Updates xlsx G31/I31 + scorecard.md log for 2c84e9c4. Held below 90
for first restore drill + fallback removal.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1811,7 +1811,7 @@
         <v>2</v>
       </c>
       <c r="G31" s="43" t="n">
-        <v>68</v>
+        <v>88</v>
       </c>
       <c r="H31" s="39">
         <f>IF(G31="","",G31*F31)</f>
@@ -1819,7 +1819,7 @@
       </c>
       <c r="I31" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: D1 schema + lazy tables; no migration story, no backups seen</t>
+          <t>Sep 16 2026: lazy gap closed (2c84e9c4) — 0015/0016, parity gates 3/3, CI auto-migrate, story doc. Residual: first restore drill (#38), runtime-fallback removal after apply proven</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: flags rows #41/#49 45/50 -> 88, composite 76.8 -> 77.8
Updates xlsx G45/I45/G53/I53 + scorecard.md log for 7141989a. Held
below 92 for rollback pipeline (per-plan deferral) + propagation
proof.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -2371,7 +2371,7 @@
         <v>1</v>
       </c>
       <c r="G45" s="43" t="n">
-        <v>45</v>
+        <v>88</v>
       </c>
       <c r="H45" s="39">
         <f>IF(G45="","",G45*F45)</f>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="I45" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: Only ad-hoc const flags (GEMINI_ENGINE_LIVE)</t>
+          <t>Sep 16 2026: flag service live (7141989a) — 0017, public+admin APIs, useFlag hook, audit-logged toggles</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
         <v>1</v>
       </c>
       <c r="G53" s="43" t="n">
-        <v>50</v>
+        <v>88</v>
       </c>
       <c r="H53" s="39">
         <f>IF(G53="","",G53*F53)</f>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="I53" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: No kill-switch; rollback = 15-min rebuild</t>
+          <t>Sep 16 2026: AI kill-switch live (7141989a) — 3 endpoints 503 pre-spend, admin UI with kill confirm, engine const migrated. Rollback pipeline deferred per plan</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: abuse row #37 85 -> 93, composite 77.8 -> 77.9
Updates xlsx G41/I41 + scorecard.md log for 08348464. Held below 96
for Turnstile-on-AI, CGNAT tuning, abuse dashboard.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -2211,7 +2211,7 @@
         <v>2</v>
       </c>
       <c r="G41" s="43" t="n">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="H41" s="39">
         <f>IF(G41="","",G41*F41)</f>
@@ -2219,7 +2219,7 @@
       </c>
       <c r="I41" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: Per-endpoint limits + Turnstile + fingerprint quotas</t>
+          <t>Sep 16 2026: layers reviewed (08348464) — dead abuse logging fixed, AI IP-velocity + anon backstop, fp index 0018, ABUSE.md. Residual: Turnstile-on-AI (covered by credits+velocity), CGNAT tuning on prod data</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: release row #20 65 -> 85, composite 77.9 -> 78.2
Updates xlsx G24/I24 + scorecard.md log for 741dc4e3. Held below 90
for first tagged release cycle.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1531,7 +1531,7 @@
         <v>1</v>
       </c>
       <c r="G24" s="43" t="n">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="H24" s="39">
         <f>IF(G24="","",G24*F24)</f>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="I24" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: Changelog exists; no semver; rollback = slow rebuild</t>
+          <t>Sep 16 2026: version truth 2.4.0 + /status display, RELEASE.md (semver/changelog/rollback), additive-migration rule (741dc4e3). Residual: first tagged release cycle</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: deps row #22 75 -> 88, composite 78.2 -> 78.3
Updates xlsx G26/I26 + scorecard.md log for 6c5ffd41. Held below
target for jspdf/pptxgenjs majors.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1611,7 +1611,7 @@
         <v>1</v>
       </c>
       <c r="G26" s="43" t="n">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="H26" s="39">
         <f>IF(G26="","",G26*F26)</f>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="I26" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: CI audit gate; MediaPipe pinned; no lockfile surprises seen</t>
+          <t>Sep 16 2026: cadence live (6c5ffd41) — next 16.3.5 build-proven, audit-ci gate green-meaningful, Dependabot weekly, ledger. Residual: jspdf/pptxgenjs majors need regression passes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: observability row #21 80 -> 90, composite 78.3 -> 78.6
Updates xlsx G25/I25 + scorecard.md log for 4d2497c9. Held below 93
for owner setup + prod-noise tuning.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1571,7 +1571,7 @@
         <v>2</v>
       </c>
       <c r="G25" s="43" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H25" s="39">
         <f>IF(G25="","",G25*F25)</f>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="I25" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: error/download/ai-credit events; admin analytics repaired Sep 12</t>
+          <t>Sep 16 2026: paging live (4d2497c9) — threshold endpoint 7/7, 15-min scheduler, Cloudflare email relay, cooldowns, runbook. Needs owner setup (domain, token, recipient). Residual: 93 needs prod-noise tuning</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: onboarding row #32 70 -> 86, composite 78.6 -> 78.8
Updates xlsx G36/I36 + scorecard.md log for a52a0963. Held below 92
for human-eyes pass + richer tour.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -2011,7 +2011,7 @@
         <v>1</v>
       </c>
       <c r="G36" s="43" t="n">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="H36" s="39">
         <f>IF(G36="","",G36*F36)</f>
@@ -2019,7 +2019,7 @@
       </c>
       <c r="I36" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: Tour per-account Sep 12; empty states guided, unverified</t>
+          <t>Sep 16 2026: empties completed + tour mobile fix + anchor gate (a52a0963); dropzone audit found coverage adequate. Residual: human-eyes pass (lab block), richer tour beyond 3 steps</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: mobile row #10 78 -> 86, composite 78.8 -> 79.0
Updates xlsx G14/I14 + scorecard.md log for 739a3879. Held below 92
for owner device audit.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1131,7 +1131,7 @@
         <v>2</v>
       </c>
       <c r="G14" s="43" t="n">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H14" s="39">
         <f>IF(G14="","",G14*F14)</f>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="I14" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: Responsive + Capacitor; PWA manifest fixed Sep 12</t>
+          <t>Sep 16 2026: offline fallback + SW wiring proven, manifest id, shortcut gate, device checklist (739a3879). Residual: owner device audit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: degraded row #45 65 -> 84, composite 79.0 -> 79.2
Updates xlsx G49/I49 + scorecard.md log for 4eb7729e. Held below 88
for live throttled verification + quota-wall-before-JS.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -2531,7 +2531,7 @@
         <v>1</v>
       </c>
       <c r="G49" s="43" t="n">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="H49" s="39">
         <f>IF(G49="","",G49*F49)</f>
@@ -2539,7 +2539,7 @@
       </c>
       <c r="I49" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: SW caches shell; CDN-first loads fragile offline</t>
+          <t>Sep 16 2026: global offline banner, offline-aware AI errors, no-auto-retry rule (4eb7729e). Residual: throttled-network live verification, quota-wall-before-JS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: energy row #47 65 -> 82, composite 79.2 -> 79.4
Updates xlsx G51/I51 + scorecard.md log for 02f7c7a5. Held below 85
for lab battery measurements.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -2611,7 +2611,7 @@
         <v>1</v>
       </c>
       <c r="G51" s="43" t="n">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="H51" s="39">
         <f>IF(G51="","",G51*F51)</f>
@@ -2619,7 +2619,7 @@
       </c>
       <c r="I51" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: Low-end detection + sequential defaults; WASM is heavy</t>
+          <t>Sep 16 2026: last unwarned engines covered + gate + ledger (02f7c7a5). Residual: lab battery measurements</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: compat row #31 75 -> 85, composite 79.4 -> 79.6
Updates xlsx G35/I35 + scorecard.md log for 9395bdf7. Held below 90
for manual device rows.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1971,7 +1971,7 @@
         <v>2</v>
       </c>
       <c r="G35" s="43" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="H35" s="39">
         <f>IF(G35="","",G35*F35)</f>
@@ -1979,7 +1979,7 @@
       </c>
       <c r="I35" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: Modern browsers OK; SAB/FFmpeg env-sensitive</t>
+          <t>Sep 16 2026: 3-engine CI matrix + baseline spec + matrix doc (9395bdf7). Residual: manual device rows, heavy-engine CI deliberately excluded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
drill#38 PASS + score 50 -> 90, composite 79.6 -> 80.6
Agent-run on owner credentials: read-only export, scratch import
(2283 rows/13 tables), per-table verification, scratch deleted.
Unwritten-path tables absent as expected at low traffic. Runtime
fallbacks stay until the CI migrate job is confirmed live.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -2251,7 +2251,7 @@
         <v>2</v>
       </c>
       <c r="G42" s="43" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="H42" s="39">
         <f>IF(G42="","",G42*F42)</f>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="I42" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: No backup/DR story found for D1</t>
+          <t>Sep 16 2026: DRILL PASS — 148KB export, 2283 rows/13 tables into scratch, all core tables queryable, scratch deleted. ai_credit_event/feature_flag/alert_log/user_flags absent = unwritten paths, not corruption</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: depth row #2 76 -> 80, composite 80.6 -> 80.7
Recounted 345/1144 with 4+ FAQs (stale note said 288); bulk5 QA
spot-check passed. Held for remaining ~800.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -811,7 +811,7 @@
         <v>3</v>
       </c>
       <c r="G6" s="43" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H6" s="39">
         <f>IF(G6="","",G6*F6)</f>
@@ -819,7 +819,7 @@
       </c>
       <c r="I6" s="40" t="inlineStr">
         <is>
-          <t>Sep 15 2026: 49 tools deepened w/ worked-example FAQs + 21 hub intros rewritten; 288/1144 w/ 4+ FAQs; tail 847 zero-custom via fallback (bulk path pending)</t>
+          <t>Sep 16 2026: 345/1144 w/ 4+ FAQs (5 gated bulk batches, pairwise-sim verified, worked examples); tail ~800 via fallback</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
counsel#26: legal review pass + action plan marked to actuals
- Entity: drop false 'Inc.' designation (terms, privacy, disclaimer,
  footer); subscriptions/billing terms mirror live behavior; 12-month
  liability cap; copyright agent; children clause; India governing law;
  changelog-noticed material changes; SLA aims not promises; cancel
  copy matches email mechanism
- ACTION-PLAN.md: Phase 1-3 marked Done/Held/Parked/Open with Sep 16
  actuals; i18n park + English-only supersede noted; honest ceiling
  repriced to ~83-84
- Score #26 90->93 (held for licensed countersign + live check)
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1771,7 +1771,7 @@
         <v>2</v>
       </c>
       <c r="G30" s="43" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H30" s="39">
         <f>IF(G30="","",G30*F30)</f>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="I30" s="40" t="inlineStr">
         <is>
-          <t>Sep 16 2026: banner placebo fixed (Decline gates PostHog/telemetry), policy audited (dca5e782), erasure cascade + 90-day purge enforced (b6055cb0). Residual: unnamed DPDP officer (owner), live prod check, lawyer review</t>
+          <t>Sep 16 2026: counsel pass — entity designation fixed, billing/subscription terms, liability cap, copyright agent, children, India governing law, SLA softening, cancel-copy fix</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: release row #20 85 -> 90, composite 80.7 -> 80.8
First tagged release cycle done (v2.5.0). Item closed.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1531,7 +1531,7 @@
         <v>1</v>
       </c>
       <c r="G24" s="43" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="H24" s="39">
         <f>IF(G24="","",G24*F24)</f>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="I24" s="40" t="inlineStr">
         <is>
-          <t>Sep 16 2026: version truth 2.4.0 + /status display, RELEASE.md (semver/changelog/rollback), additive-migration rule (741dc4e3). Residual: first tagged release cycle</t>
+          <t>Sep 16 2026: v2.5.0 tagged + pushed, changelog entry, /status reads version — first cycle complete</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
build#15: measured pipeline, documented headroom, scored 72->78
gen steps ~7s, OG incremental ~11s, compile+static already at
hardware parallelism. BUILD.md ledger + no-dirty-tree rule.
Held below 86: remaining is hardware or page-count scope.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1331,7 +1331,7 @@
         <v>2</v>
       </c>
       <c r="G19" s="43" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="H19" s="39">
         <f>IF(G19="","",G19*F19)</f>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="I19" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: 15-min builds hurt; bundles cut 30-35%; OG decoupled</t>
+          <t>Sep 16 2026: measured, not assumed — pipeline already parallel/incremental/cached; BUILD.md ledger + hygiene rule (remaining is hardware)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: load row #42 40 -> 65, composite 81.0 -> 81.3
Rig armed, unfired by rule (e30e6f8c). Held for first fired run.
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -2411,7 +2411,7 @@
         <v>1</v>
       </c>
       <c r="G46" s="43" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="H46" s="39">
         <f>IF(G46="","",G46*F46)</f>
@@ -2419,7 +2419,7 @@
       </c>
       <c r="I46" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: No load/stress testing seen</t>
+          <t>Sep 16 2026: rig armed, unfired by rule (e30e6f8c) — scenarios, prod guard, checker, manual CI, 10x trigger. No proof yet by design</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scorecard: auth row #25 82 -> 90, composite 81.3 -> 81.5
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1731,7 +1731,7 @@
         <v>2</v>
       </c>
       <c r="G29" s="43" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="H29" s="39">
         <f>IF(G29="","",G29*F29)</f>
@@ -1739,7 +1739,7 @@
       </c>
       <c r="I29" s="40" t="inlineStr">
         <is>
-          <t>Sep 12 2026: better-auth Google+email; sessions; admin roles; login saga fixed</t>
+          <t>Sep 17 2026: D1 auth throttle + full review (ae258587); admin audit complete. Residual: login CAPTCHA escalation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: scorecard updates — exclude N/A items (i18n, team, platform, experimentation), #33 to 65
</commit_message>
<xml_diff>
--- a/docs/ToolZum- App_Production_Scorecard_51.xlsx
+++ b/docs/ToolZum- App_Production_Scorecard_51.xlsx
@@ -1930,9 +1930,7 @@
       <c r="F34" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="G34" s="43" t="n">
-        <v>35</v>
-      </c>
+      <c r="G34" s="43" t="n"/>
       <c r="H34" s="39">
         <f>IF(G34="","",G34*F34)</f>
         <v/>
@@ -2051,7 +2049,7 @@
         <v>1</v>
       </c>
       <c r="G37" s="43" t="n">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="H37" s="39">
         <f>IF(G37="","",G37*F37)</f>
@@ -2330,9 +2328,7 @@
       <c r="F44" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="G44" s="43" t="n">
-        <v>40</v>
-      </c>
+      <c r="G44" s="43" t="n"/>
       <c r="H44" s="39">
         <f>IF(G44="","",G44*F44)</f>
         <v/>
@@ -2570,9 +2566,7 @@
       <c r="F50" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="G50" s="43" t="n">
-        <v>55</v>
-      </c>
+      <c r="G50" s="43" t="n"/>
       <c r="H50" s="39">
         <f>IF(G50="","",G50*F50)</f>
         <v/>
@@ -2650,9 +2644,7 @@
       <c r="F52" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="G52" s="43" t="n">
-        <v>30</v>
-      </c>
+      <c r="G52" s="43" t="n"/>
       <c r="H52" s="39">
         <f>IF(G52="","",G52*F52)</f>
         <v/>
@@ -2730,9 +2722,7 @@
       <c r="F54" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="G54" s="43" t="n">
-        <v>20</v>
-      </c>
+      <c r="G54" s="43" t="n"/>
       <c r="H54" s="39">
         <f>IF(G54="","",G54*F54)</f>
         <v/>

</xml_diff>